<commit_message>
Freeze final reproduction results and integrity records
</commit_message>
<xml_diff>
--- a/results/primary/primary_tables.xlsx
+++ b/results/primary/primary_tables.xlsx
@@ -478,13 +478,13 @@
         <v>0.8430605421970768</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4014355539839699</v>
+        <v>0.4023419000471476</v>
       </c>
       <c r="D2" t="n">
-        <v>7.994891267457727</v>
+        <v>8.018367429330237</v>
       </c>
       <c r="E2" t="n">
-        <v>9.749182963018002</v>
+        <v>9.777962963213362</v>
       </c>
       <c r="F2" t="n">
         <v>0.8925555126984127</v>
@@ -509,13 +509,13 @@
         <v>0.861754912776992</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1920292597831212</v>
+        <v>0.1918875058934465</v>
       </c>
       <c r="D3" t="n">
-        <v>3.141675175203496</v>
+        <v>3.141357003318696</v>
       </c>
       <c r="E3" t="n">
-        <v>3.965885756750486</v>
+        <v>3.965731277548442</v>
       </c>
       <c r="F3" t="n">
         <v>0.8547992206349208</v>
@@ -540,13 +540,13 @@
         <v>0.8066516030174445</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2048616218764734</v>
+        <v>0.2050022347949081</v>
       </c>
       <c r="D4" t="n">
-        <v>3.282579717615958</v>
+        <v>3.282222450941116</v>
       </c>
       <c r="E4" t="n">
-        <v>4.295359255708684</v>
+        <v>4.295603008022032</v>
       </c>
       <c r="F4" t="n">
         <v>0.8472197968253968</v>
@@ -571,13 +571,13 @@
         <v>0.8384317444601603</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2084848326261197</v>
+        <v>0.2085786468646865</v>
       </c>
       <c r="D5" t="n">
-        <v>3.294692601156781</v>
+        <v>3.296760862643964</v>
       </c>
       <c r="E5" t="n">
-        <v>4.495417191845697</v>
+        <v>4.498278550124857</v>
       </c>
       <c r="F5" t="n">
         <v>0.8313204333333334</v>
@@ -602,13 +602,13 @@
         <v>0.9240068646864686</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2828240735502122</v>
+        <v>0.2864720179160773</v>
       </c>
       <c r="D6" t="n">
-        <v>5.053252176240659</v>
+        <v>5.085344674400394</v>
       </c>
       <c r="E6" t="n">
-        <v>6.367819216025069</v>
+        <v>6.404212382650993</v>
       </c>
       <c r="F6" t="n">
         <v>0.8920220555555556</v>

</xml_diff>